<commit_message>
Enter Source Metals invoices 470223 and 470471 on batch 749.
The Fabcorp scans are vendor 338. Both bills are unposted, balanced with freight, and the emails are archived.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/sept-missed-entry-2026-10-07/AP-sept-missed-2026-10-07.xlsx
+++ b/runs/sept-missed-entry-2026-10-07/AP-sept-missed-2026-10-07.xlsx
@@ -999,7 +999,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fabcorp</t>
+          <t>Source Metals</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1008,12 +1008,14 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2280</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+        <v>1625</v>
+      </c>
+      <c r="D15" t="n">
+        <v>10539</v>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1023,20 +1025,22 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The scan total is $2,280.00. PO 59060 is a Source Metals purchase order, and Fabcorp has no KIMCO vendor id, so no bill was created.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>PO 59060 receipts 24175, 24176, 24177, 24178, 24181, and 24182 are 12 pieces of the 1.25 plate at $95.00, $1,140.00. Receipts 24184, 24185, and 24186 are 6 pieces at $20.00, $120.00. Receipts 24179, 24180, and 24183 are 6 pieces at $15.00, $90.00. The unit is each on the invoice and the receipts. Freight $275.00 is Freight External. There is no price variance.</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1733</v>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>y</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fabcorp</t>
+          <t>Source Metals</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1045,12 +1049,14 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>330</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>1335</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10540</v>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1060,13 +1066,15 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The scan total is $330.00. PO 59216 is a Source Metals purchase order, and Fabcorp has no KIMCO vendor id, so no bill was created.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>PO 59216 receipt 25258 is 4 pieces at $262.50, $1,050.00. The unit is each on the invoice and the receipt. Freight $285.00 is Freight External. There is no price variance.</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>1734</v>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>y</t>
         </is>
       </c>
     </row>

</xml_diff>